<commit_message>
Still need to fix FM beta arg
</commit_message>
<xml_diff>
--- a/Indicator_4/Real_data/Blue_Shark_IO.xlsx
+++ b/Indicator_4/Real_data/Blue_Shark_IO.xlsx
@@ -1,294 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\EcoTest_Train\Indicator_4\Real_data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A2926F-72E2-4E4D-AB9A-0D408FCA20A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="Time_series" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="87">
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Blue_Shark_IO</t>
-  </si>
-  <si>
-    <t>E.g. 'Swordfish_Natl'</t>
-  </si>
-  <si>
-    <t>Stock</t>
-  </si>
-  <si>
-    <t>max_age</t>
-  </si>
-  <si>
-    <t>18.446</t>
-  </si>
-  <si>
-    <t>Age to 5% natural survival</t>
-  </si>
-  <si>
-    <t>Life history</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>0.129</t>
-  </si>
-  <si>
-    <t>von Bertalannfy K</t>
-  </si>
-  <si>
-    <t>Linf</t>
-  </si>
-  <si>
-    <t>0.512</t>
-  </si>
-  <si>
-    <t>von Bertalannfy L-infinity (asymptotic length)</t>
-  </si>
-  <si>
-    <t>L50_Linf</t>
-  </si>
-  <si>
-    <t>283.2</t>
-  </si>
-  <si>
-    <t>Length at 50% maturity relative to asymptotic length (von B. L-infinity)</t>
-  </si>
-  <si>
-    <t>Total_L5_L50</t>
-  </si>
-  <si>
-    <t>0.741</t>
-  </si>
-  <si>
-    <t>Length at 5% selection relative to length at 50% maturity</t>
-  </si>
-  <si>
-    <t>Fleet selectivity</t>
-  </si>
-  <si>
-    <t>All fleets combined</t>
-  </si>
-  <si>
-    <t>Total_LFS_L50</t>
-  </si>
-  <si>
-    <t>1.534</t>
-  </si>
-  <si>
-    <t>Length at full selection relative to length at 50% maturity</t>
-  </si>
-  <si>
-    <t>Total_VML</t>
-  </si>
-  <si>
-    <t>0.97</t>
-  </si>
-  <si>
-    <t>Selectivity of maximum length class</t>
-  </si>
-  <si>
-    <t>Fleet_1_L5_L50</t>
-  </si>
-  <si>
-    <t>0.325</t>
-  </si>
-  <si>
-    <t>Fleet 1</t>
-  </si>
-  <si>
-    <t>Fleet_1_LFS_L50</t>
-  </si>
-  <si>
-    <t>1.027</t>
-  </si>
-  <si>
-    <t>Fleet_1_VML</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Fleet_2_L5_L50</t>
-  </si>
-  <si>
-    <t>0.734</t>
-  </si>
-  <si>
-    <t>Fleet 2</t>
-  </si>
-  <si>
-    <t>Fleet_2_LFS_L50</t>
-  </si>
-  <si>
-    <t>1.303</t>
-  </si>
-  <si>
-    <t>Fleet_2_VML</t>
-  </si>
-  <si>
-    <t>Fleet_3_L5_L50</t>
-  </si>
-  <si>
-    <t>0.826</t>
-  </si>
-  <si>
-    <t>Fleet 3</t>
-  </si>
-  <si>
-    <t>Fleet_3_LFS_L50</t>
-  </si>
-  <si>
-    <t>1.678</t>
-  </si>
-  <si>
-    <t>Fleet_3_VML</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Fleet_1_CF</t>
-  </si>
-  <si>
-    <t>0.092</t>
-  </si>
-  <si>
-    <t>Fraction of all historical catches that were Fleet 1</t>
-  </si>
-  <si>
-    <t>Fleet catch scale</t>
-  </si>
-  <si>
-    <t>Fleet_2_CF</t>
-  </si>
-  <si>
-    <t>Fraction of all historical catches that were Fleet 2</t>
-  </si>
-  <si>
-    <t>Fleet_3_CF</t>
-  </si>
-  <si>
-    <t>0.816</t>
-  </si>
-  <si>
-    <t>Fraction of all historical catches that were Fleet 3</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Total_catch</t>
-  </si>
-  <si>
-    <t>Total_mean_len</t>
-  </si>
-  <si>
-    <t>Total_mean_age</t>
-  </si>
-  <si>
-    <t>Total_CV_len</t>
-  </si>
-  <si>
-    <t>Total_frac_mat</t>
-  </si>
-  <si>
-    <t>Total_Index</t>
-  </si>
-  <si>
-    <t>Fleet_1_catch</t>
-  </si>
-  <si>
-    <t>Fleet_1_mean_len</t>
-  </si>
-  <si>
-    <t>Fleet_1_mean_age</t>
-  </si>
-  <si>
-    <t>Fleet_1_CV_len</t>
-  </si>
-  <si>
-    <t>Fleet_1_frac_mat</t>
-  </si>
-  <si>
-    <t>Fleet_1_Index</t>
-  </si>
-  <si>
-    <t>Fleet_2_catch</t>
-  </si>
-  <si>
-    <t>Fleet_2_mean_len</t>
-  </si>
-  <si>
-    <t>Fleet_2_mean_age</t>
-  </si>
-  <si>
-    <t>Fleet_2_CV_len</t>
-  </si>
-  <si>
-    <t>Fleet_2_frac_mat</t>
-  </si>
-  <si>
-    <t>Fleet_2_Index</t>
-  </si>
-  <si>
-    <t>Fleet_3_catch</t>
-  </si>
-  <si>
-    <t>Fleet_3_mean_len</t>
-  </si>
-  <si>
-    <t>Fleet_3_mean_age</t>
-  </si>
-  <si>
-    <t>Fleet_3_CV_len</t>
-  </si>
-  <si>
-    <t>Fleet_3_frac_mat</t>
-  </si>
-  <si>
-    <t>Fleet_3_Index</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,21 +64,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -388,7 +108,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -422,7 +142,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -457,10 +176,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -633,365 +351,575 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B20" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" t="s">
-        <v>56</v>
-      </c>
-      <c r="E21" t="s">
-        <v>48</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blue_Shark_IO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E.g. 'Swordfish_Natl'</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>max_age</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>18.446</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Age to 5% natural survival</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Life history</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0.129</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>von Bertalannfy K</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Life history</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Linf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.512</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>von Bertalannfy L-infinity (asymptotic length)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Life history</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L50_Linf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>283.2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Length at 50% maturity relative to asymptotic length (von B. L-infinity)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Life history</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total_L5_L50</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.741</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Length at 5% selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>All fleets combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Total_LFS_L50</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1.534</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Length at full selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>All fleets combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total_VML</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Selectivity of maximum length class</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>All fleets combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fleet_1_L5_L50</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.325</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Length at 5% selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fleet 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fleet_1_LFS_L50</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1.027</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Length at full selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fleet 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fleet_1_VML</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Selectivity of maximum length class</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Fleet 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fleet_2_L5_L50</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0.734</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Length at 5% selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Fleet 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fleet_2_LFS_L50</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1.303</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Length at full selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Fleet 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fleet_2_VML</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Selectivity of maximum length class</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Fleet 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fleet_3_L5_L50</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.826</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Length at 5% selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Fleet 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Fleet_3_LFS_L50</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1.678</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Length at full selection relative to length at 50% maturity</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Fleet 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fleet_3_VML</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Selectivity of maximum length class</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fleet selectivity</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Fleet 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Fleet_1_CF</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.092</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fraction of all historical catches that were Fleet 1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Fleet catch scale</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Fleet 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fleet_2_CF</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0.092</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fraction of all historical catches that were Fleet 2</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Fleet catch scale</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Fleet 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fleet_3_CF</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0.816</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Fraction of all historical catches that were Fleet 3</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fleet catch scale</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Fleet 3</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1000,88 +928,138 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Y71"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total_catch</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total_mean_len</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Total_mean_age</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total_CV_len</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total_frac_mat</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Index</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_catch</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_mean_len</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_mean_age</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_CV_len</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_frac_mat</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_1_Index</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_catch</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_mean_len</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_mean_age</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_CV_len</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_frac_mat</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_2_Index</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_catch</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_mean_len</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_mean_age</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_CV_len</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_frac_mat</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Fleet_3_Index</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2">
         <v>1950</v>
       </c>
@@ -1089,7 +1067,7 @@
         <v>131.691</v>
       </c>
       <c r="G2">
-        <v>1.2210000000000001</v>
+        <v>1.221</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1101,7 +1079,7 @@
         <v>131.691</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="A3">
         <v>1951</v>
       </c>
@@ -1121,12 +1099,12 @@
         <v>754.221</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4">
         <v>1952</v>
       </c>
       <c r="B4">
-        <v>1707.8330000000001</v>
+        <v>1707.833</v>
       </c>
       <c r="G4">
         <v>1.22</v>
@@ -1138,10 +1116,10 @@
         <v>0</v>
       </c>
       <c r="T4">
-        <v>821.83299999999997</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+        <v>821.833</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5">
         <v>1953</v>
       </c>
@@ -1158,15 +1136,15 @@
         <v>0</v>
       </c>
       <c r="T5">
-        <v>831.70399999999995</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+        <v>831.704</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6">
         <v>1954</v>
       </c>
       <c r="B6">
-        <v>3933.6790000000001</v>
+        <v>3933.679</v>
       </c>
       <c r="G6">
         <v>1.22</v>
@@ -1178,15 +1156,15 @@
         <v>0</v>
       </c>
       <c r="T6">
-        <v>1102.6790000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1102.679</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7">
         <v>1955</v>
       </c>
       <c r="B7">
-        <v>4394.2849999999999</v>
+        <v>4394.285</v>
       </c>
       <c r="G7">
         <v>1.216</v>
@@ -1198,10 +1176,10 @@
         <v>0</v>
       </c>
       <c r="T7">
-        <v>1132.2850000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1132.285</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8">
         <v>1956</v>
       </c>
@@ -1209,7 +1187,7 @@
         <v>4051.817</v>
       </c>
       <c r="G8">
-        <v>1.2110000000000001</v>
+        <v>1.211</v>
       </c>
       <c r="H8">
         <v>2788</v>
@@ -1221,15 +1199,15 @@
         <v>1263.817</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="9">
       <c r="A9">
         <v>1957</v>
       </c>
       <c r="B9">
-        <v>4951.7619999999997</v>
+        <v>4951.762</v>
       </c>
       <c r="G9">
-        <v>1.1990000000000001</v>
+        <v>1.199</v>
       </c>
       <c r="H9">
         <v>3673</v>
@@ -1238,18 +1216,18 @@
         <v>0</v>
       </c>
       <c r="T9">
-        <v>1278.7619999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1278.762</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10">
         <v>1958</v>
       </c>
       <c r="B10">
-        <v>4791.3789999999999</v>
+        <v>4791.379</v>
       </c>
       <c r="G10">
-        <v>1.1850000000000001</v>
+        <v>1.185</v>
       </c>
       <c r="H10">
         <v>3293</v>
@@ -1258,15 +1236,15 @@
         <v>0</v>
       </c>
       <c r="T10">
-        <v>1498.3789999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1498.379</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11">
         <v>1959</v>
       </c>
       <c r="B11">
-        <v>5024.2539999999999</v>
+        <v>5024.254</v>
       </c>
       <c r="G11">
         <v>1.173</v>
@@ -1278,18 +1256,18 @@
         <v>0</v>
       </c>
       <c r="T11">
-        <v>1674.2539999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1674.254</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12">
         <v>1960</v>
       </c>
       <c r="B12">
-        <v>4587.0129999999999</v>
+        <v>4587.013</v>
       </c>
       <c r="G12">
-        <v>1.1579999999999999</v>
+        <v>1.158</v>
       </c>
       <c r="H12">
         <v>3023</v>
@@ -1298,15 +1276,15 @@
         <v>0</v>
       </c>
       <c r="T12">
-        <v>1564.0129999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1564.013</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13">
         <v>1961</v>
       </c>
       <c r="B13">
-        <v>4508.3549999999996</v>
+        <v>4508.355</v>
       </c>
       <c r="G13">
         <v>1.145</v>
@@ -1321,12 +1299,12 @@
         <v>2064.355</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="14">
       <c r="A14">
         <v>1962</v>
       </c>
       <c r="B14">
-        <v>4944.6790000000001</v>
+        <v>4944.679</v>
       </c>
       <c r="G14">
         <v>1.133</v>
@@ -1338,18 +1316,18 @@
         <v>0</v>
       </c>
       <c r="T14">
-        <v>2154.6790000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+        <v>2154.679</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15">
         <v>1963</v>
       </c>
       <c r="B15">
-        <v>5859.4170000000004</v>
+        <v>5859.417</v>
       </c>
       <c r="G15">
-        <v>1.1220000000000001</v>
+        <v>1.122</v>
       </c>
       <c r="H15">
         <v>3507</v>
@@ -1358,15 +1336,15 @@
         <v>0</v>
       </c>
       <c r="T15">
-        <v>2352.4169999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+        <v>2352.417</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16">
         <v>1964</v>
       </c>
       <c r="B16">
-        <v>6521.1850000000004</v>
+        <v>6521.185</v>
       </c>
       <c r="G16">
         <v>1.115</v>
@@ -1378,15 +1356,15 @@
         <v>0</v>
       </c>
       <c r="T16">
-        <v>2023.1849999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
+        <v>2023.185</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17">
         <v>1965</v>
       </c>
       <c r="B17">
-        <v>4479.4859999999999</v>
+        <v>4479.486</v>
       </c>
       <c r="G17">
         <v>1.107</v>
@@ -1398,15 +1376,15 @@
         <v>0</v>
       </c>
       <c r="T17">
-        <v>1399.4860000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1399.486</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18">
         <v>1966</v>
       </c>
       <c r="B18">
-        <v>5472.7790000000005</v>
+        <v>5472.779</v>
       </c>
       <c r="G18">
         <v>1.097</v>
@@ -1421,12 +1399,12 @@
         <v>2494.779</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="19">
       <c r="A19">
         <v>1967</v>
       </c>
       <c r="B19">
-        <v>8939.8160000000007</v>
+        <v>8939.816000000001</v>
       </c>
       <c r="G19">
         <v>1.085</v>
@@ -1438,18 +1416,18 @@
         <v>0</v>
       </c>
       <c r="T19">
-        <v>4595.8159999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
+        <v>4595.816</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20">
         <v>1968</v>
       </c>
       <c r="B20">
-        <v>8621.1470000000008</v>
+        <v>8621.147000000001</v>
       </c>
       <c r="G20">
-        <v>1.0780000000000001</v>
+        <v>1.078</v>
       </c>
       <c r="H20">
         <v>3384</v>
@@ -1458,15 +1436,15 @@
         <v>0</v>
       </c>
       <c r="T20">
-        <v>5237.1469999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
+        <v>5237.147</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21">
         <v>1969</v>
       </c>
       <c r="B21">
-        <v>9030.3420000000006</v>
+        <v>9030.342000000001</v>
       </c>
       <c r="G21">
         <v>1.071</v>
@@ -1478,18 +1456,18 @@
         <v>0</v>
       </c>
       <c r="T21">
-        <v>5639.3419999999996</v>
-      </c>
-    </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
+        <v>5639.342</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="A22">
         <v>1970</v>
       </c>
       <c r="B22">
-        <v>4842.0590000000002</v>
+        <v>4842.059</v>
       </c>
       <c r="G22">
-        <v>1.0569999999999999</v>
+        <v>1.057</v>
       </c>
       <c r="H22">
         <v>2106</v>
@@ -1498,15 +1476,15 @@
         <v>0</v>
       </c>
       <c r="T22">
-        <v>2736.0590000000002</v>
-      </c>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
+        <v>2736.059</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23">
         <v>1971</v>
       </c>
       <c r="B23">
-        <v>5165.5290000000005</v>
+        <v>5165.529</v>
       </c>
       <c r="G23">
         <v>1.046</v>
@@ -1521,10 +1499,10 @@
         <v>3006.529</v>
       </c>
       <c r="Y23">
-        <v>1.0720000000000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.072</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24">
         <v>1972</v>
       </c>
@@ -1544,15 +1522,15 @@
         <v>3374.607</v>
       </c>
       <c r="Y24">
-        <v>1.0720000000000001</v>
-      </c>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.072</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25">
         <v>1973</v>
       </c>
       <c r="B25">
-        <v>3385.0639999999999</v>
+        <v>3385.064</v>
       </c>
       <c r="G25">
         <v>1.032</v>
@@ -1564,18 +1542,18 @@
         <v>0</v>
       </c>
       <c r="T25">
-        <v>2515.0639999999999</v>
+        <v>2515.064</v>
       </c>
       <c r="Y25">
-        <v>0.76800000000000002</v>
-      </c>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26">
         <v>1974</v>
       </c>
       <c r="B26">
-        <v>5004.5540000000001</v>
+        <v>5004.554</v>
       </c>
       <c r="G26">
         <v>1.03</v>
@@ -1587,21 +1565,21 @@
         <v>0</v>
       </c>
       <c r="T26">
-        <v>3671.5540000000001</v>
+        <v>3671.554</v>
       </c>
       <c r="Y26">
-        <v>1.2070000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.207</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27">
         <v>1975</v>
       </c>
       <c r="B27">
-        <v>5399.7269999999999</v>
+        <v>5399.727</v>
       </c>
       <c r="G27">
-        <v>1.0309999999999999</v>
+        <v>1.031</v>
       </c>
       <c r="H27">
         <v>1191</v>
@@ -1610,21 +1588,21 @@
         <v>0</v>
       </c>
       <c r="T27">
-        <v>4208.7269999999999</v>
+        <v>4208.727</v>
       </c>
       <c r="Y27">
-        <v>1.4510000000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.451</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28">
         <v>1976</v>
       </c>
       <c r="B28">
-        <v>4636.0339999999997</v>
+        <v>4636.034</v>
       </c>
       <c r="G28">
-        <v>1.0369999999999999</v>
+        <v>1.037</v>
       </c>
       <c r="H28">
         <v>473</v>
@@ -1633,13 +1611,13 @@
         <v>0</v>
       </c>
       <c r="T28">
-        <v>4163.0339999999997</v>
+        <v>4163.034</v>
       </c>
       <c r="Y28">
-        <v>1.0289999999999999</v>
-      </c>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.029</v>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29">
         <v>1977</v>
       </c>
@@ -1647,7 +1625,7 @@
         <v>5048.116</v>
       </c>
       <c r="G29">
-        <v>1.0389999999999999</v>
+        <v>1.039</v>
       </c>
       <c r="H29">
         <v>439</v>
@@ -1659,15 +1637,15 @@
         <v>4609.116</v>
       </c>
       <c r="Y29">
-        <v>1.3420000000000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.342</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30">
         <v>1978</v>
       </c>
       <c r="B30">
-        <v>6252.3329999999996</v>
+        <v>6252.333</v>
       </c>
       <c r="G30">
         <v>1.042</v>
@@ -1679,21 +1657,21 @@
         <v>0</v>
       </c>
       <c r="T30">
-        <v>5487.3329999999996</v>
+        <v>5487.333</v>
       </c>
       <c r="Y30">
-        <v>0.77600000000000002</v>
-      </c>
-    </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.776</v>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31">
         <v>1979</v>
       </c>
       <c r="B31">
-        <v>7963.2719999999999</v>
+        <v>7963.272</v>
       </c>
       <c r="G31">
-        <v>1.0469999999999999</v>
+        <v>1.047</v>
       </c>
       <c r="H31">
         <v>895</v>
@@ -1702,18 +1680,18 @@
         <v>0</v>
       </c>
       <c r="T31">
-        <v>7068.2719999999999</v>
+        <v>7068.272</v>
       </c>
       <c r="Y31">
-        <v>1.2490000000000001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.249</v>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32">
         <v>1980</v>
       </c>
       <c r="B32">
-        <v>7532.7960000000003</v>
+        <v>7532.796</v>
       </c>
       <c r="G32">
         <v>1.052</v>
@@ -1725,18 +1703,18 @@
         <v>0</v>
       </c>
       <c r="T32">
-        <v>6644.7960000000003</v>
+        <v>6644.796</v>
       </c>
       <c r="Y32">
         <v>1.046</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="33">
       <c r="A33">
         <v>1981</v>
       </c>
       <c r="B33">
-        <v>10300.058000000001</v>
+        <v>10300.058</v>
       </c>
       <c r="G33">
         <v>1.056</v>
@@ -1748,18 +1726,18 @@
         <v>0</v>
       </c>
       <c r="T33">
-        <v>9193.0580000000009</v>
+        <v>9193.058000000001</v>
       </c>
       <c r="Y33">
-        <v>0.98699999999999999</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.987</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34">
         <v>1982</v>
       </c>
       <c r="B34">
-        <v>9447.5830000000005</v>
+        <v>9447.583000000001</v>
       </c>
       <c r="G34">
         <v>1.056</v>
@@ -1771,13 +1749,13 @@
         <v>0</v>
       </c>
       <c r="T34">
-        <v>8625.5830000000005</v>
+        <v>8625.583000000001</v>
       </c>
       <c r="Y34">
         <v>1.409</v>
       </c>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="35">
       <c r="A35">
         <v>1983</v>
       </c>
@@ -1785,7 +1763,7 @@
         <v>10959.38</v>
       </c>
       <c r="G35">
-        <v>1.0569999999999999</v>
+        <v>1.057</v>
       </c>
       <c r="H35">
         <v>1076</v>
@@ -1794,18 +1772,18 @@
         <v>0</v>
       </c>
       <c r="T35">
-        <v>9883.3799999999992</v>
+        <v>9883.379999999999</v>
       </c>
       <c r="Y35">
-        <v>0.83499999999999996</v>
-      </c>
-    </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.835</v>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36">
         <v>1984</v>
       </c>
       <c r="B36">
-        <v>11314.789000000001</v>
+        <v>11314.789</v>
       </c>
       <c r="G36">
         <v>1.054</v>
@@ -1817,18 +1795,18 @@
         <v>0</v>
       </c>
       <c r="T36">
-        <v>10121.789000000001</v>
+        <v>10121.789</v>
       </c>
       <c r="Y36">
         <v>1.147</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="37">
       <c r="A37">
         <v>1985</v>
       </c>
       <c r="B37">
-        <v>7028.1589999999997</v>
+        <v>7028.159</v>
       </c>
       <c r="G37">
         <v>1.054</v>
@@ -1840,18 +1818,18 @@
         <v>0</v>
       </c>
       <c r="T37">
-        <v>6015.1589999999997</v>
+        <v>6015.159</v>
       </c>
       <c r="Y37">
-        <v>1.0549999999999999</v>
-      </c>
-    </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.055</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38">
         <v>1986</v>
       </c>
       <c r="B38">
-        <v>9807.1119999999992</v>
+        <v>9807.111999999999</v>
       </c>
       <c r="G38">
         <v>1.052</v>
@@ -1863,21 +1841,21 @@
         <v>0</v>
       </c>
       <c r="T38">
-        <v>8706.1119999999992</v>
+        <v>8706.111999999999</v>
       </c>
       <c r="Y38">
-        <v>0.97899999999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.979</v>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39">
         <v>1987</v>
       </c>
       <c r="B39">
-        <v>9068.11</v>
+        <v>9068.110000000001</v>
       </c>
       <c r="G39">
-        <v>1.0489999999999999</v>
+        <v>1.049</v>
       </c>
       <c r="H39">
         <v>953</v>
@@ -1889,18 +1867,18 @@
         <v>8115.11</v>
       </c>
       <c r="Y39">
-        <v>0.93700000000000006</v>
-      </c>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.9370000000000001</v>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40">
         <v>1988</v>
       </c>
       <c r="B40">
-        <v>10414.316000000001</v>
+        <v>10414.316</v>
       </c>
       <c r="G40">
-        <v>1.0509999999999999</v>
+        <v>1.051</v>
       </c>
       <c r="H40">
         <v>848</v>
@@ -1909,18 +1887,18 @@
         <v>0</v>
       </c>
       <c r="T40">
-        <v>9566.3160000000007</v>
+        <v>9566.316000000001</v>
       </c>
       <c r="Y40">
         <v>1.131</v>
       </c>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="41">
       <c r="A41">
         <v>1989</v>
       </c>
       <c r="B41">
-        <v>13167.272000000001</v>
+        <v>13167.272</v>
       </c>
       <c r="G41">
         <v>1.048</v>
@@ -1932,18 +1910,18 @@
         <v>0</v>
       </c>
       <c r="T41">
-        <v>12519.272000000001</v>
+        <v>12519.272</v>
       </c>
       <c r="Y41">
         <v>1.004</v>
       </c>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="42">
       <c r="A42">
         <v>1990</v>
       </c>
       <c r="B42">
-        <v>8256.2939999999999</v>
+        <v>8256.294</v>
       </c>
       <c r="G42">
         <v>1.044</v>
@@ -1955,21 +1933,21 @@
         <v>0</v>
       </c>
       <c r="T42">
-        <v>7767.2939999999999</v>
+        <v>7767.294</v>
       </c>
       <c r="Y42">
-        <v>1.3919999999999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.392</v>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43">
         <v>1991</v>
       </c>
       <c r="B43">
-        <v>10487.235000000001</v>
+        <v>10487.235</v>
       </c>
       <c r="G43">
-        <v>1.0369999999999999</v>
+        <v>1.037</v>
       </c>
       <c r="H43">
         <v>660</v>
@@ -1978,13 +1956,13 @@
         <v>0</v>
       </c>
       <c r="T43">
-        <v>9827.2350000000006</v>
+        <v>9827.235000000001</v>
       </c>
       <c r="Y43">
         <v>1.038</v>
       </c>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="44">
       <c r="A44">
         <v>1992</v>
       </c>
@@ -1995,7 +1973,7 @@
         <v>128.506</v>
       </c>
       <c r="E44">
-        <v>0.29599999999999999</v>
+        <v>0.296</v>
       </c>
       <c r="F44">
         <v>0.373</v>
@@ -2010,7 +1988,7 @@
         <v>128.506</v>
       </c>
       <c r="K44">
-        <v>0.29599999999999999</v>
+        <v>0.296</v>
       </c>
       <c r="L44">
         <v>0.373</v>
@@ -2025,10 +2003,10 @@
         <v>10227.145</v>
       </c>
       <c r="Y44">
-        <v>0.91100000000000003</v>
-      </c>
-    </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.911</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45">
         <v>1993</v>
       </c>
@@ -2039,13 +2017,13 @@
         <v>127.28</v>
       </c>
       <c r="E45">
-        <v>0.35799999999999998</v>
+        <v>0.358</v>
       </c>
       <c r="F45">
-        <v>0.40400000000000003</v>
+        <v>0.404</v>
       </c>
       <c r="G45">
-        <v>1.0169999999999999</v>
+        <v>1.017</v>
       </c>
       <c r="H45">
         <v>583</v>
@@ -2054,13 +2032,13 @@
         <v>127.28</v>
       </c>
       <c r="K45">
-        <v>0.35799999999999998</v>
+        <v>0.358</v>
       </c>
       <c r="L45">
-        <v>0.40400000000000003</v>
+        <v>0.404</v>
       </c>
       <c r="M45">
-        <v>0.55400000000000005</v>
+        <v>0.554</v>
       </c>
       <c r="N45">
         <v>52</v>
@@ -2072,24 +2050,24 @@
         <v>1.375</v>
       </c>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="46">
       <c r="A46">
         <v>1994</v>
       </c>
       <c r="B46">
-        <v>17067.864000000001</v>
+        <v>17067.864</v>
       </c>
       <c r="C46">
         <v>121.733</v>
       </c>
       <c r="E46">
-        <v>0.28999999999999998</v>
+        <v>0.29</v>
       </c>
       <c r="F46">
-        <v>0.29699999999999999</v>
+        <v>0.297</v>
       </c>
       <c r="G46">
-        <v>1.0029999999999999</v>
+        <v>1.003</v>
       </c>
       <c r="H46">
         <v>933</v>
@@ -2098,10 +2076,10 @@
         <v>121.733</v>
       </c>
       <c r="K46">
-        <v>0.28999999999999998</v>
+        <v>0.29</v>
       </c>
       <c r="L46">
-        <v>0.29699999999999999</v>
+        <v>0.297</v>
       </c>
       <c r="M46">
         <v>0.627</v>
@@ -2113,48 +2091,48 @@
         <v>15837.864</v>
       </c>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="47">
       <c r="A47">
         <v>1995</v>
       </c>
       <c r="B47">
-        <v>17570.996999999999</v>
+        <v>17570.997</v>
       </c>
       <c r="C47">
-        <v>138.86500000000001</v>
+        <v>138.865</v>
       </c>
       <c r="E47">
-        <v>0.20599999999999999</v>
+        <v>0.206</v>
       </c>
       <c r="F47">
         <v>0.38</v>
       </c>
       <c r="G47">
-        <v>0.98599999999999999</v>
+        <v>0.986</v>
       </c>
       <c r="H47">
         <v>1410</v>
       </c>
       <c r="I47">
-        <v>138.86500000000001</v>
+        <v>138.865</v>
       </c>
       <c r="K47">
-        <v>0.20599999999999999</v>
+        <v>0.206</v>
       </c>
       <c r="L47">
         <v>0.38</v>
       </c>
       <c r="M47">
-        <v>0.70299999999999996</v>
+        <v>0.703</v>
       </c>
       <c r="N47">
         <v>90</v>
       </c>
       <c r="T47">
-        <v>16070.996999999999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
+        <v>16070.997</v>
+      </c>
+    </row>
+    <row r="48">
       <c r="A48">
         <v>1996</v>
       </c>
@@ -2165,13 +2143,13 @@
         <v>127.04</v>
       </c>
       <c r="E48">
-        <v>0.28199999999999997</v>
+        <v>0.282</v>
       </c>
       <c r="F48">
-        <v>0.34499999999999997</v>
+        <v>0.345</v>
       </c>
       <c r="G48">
-        <v>0.96599999999999997</v>
+        <v>0.966</v>
       </c>
       <c r="H48">
         <v>1329</v>
@@ -2180,13 +2158,13 @@
         <v>127.04</v>
       </c>
       <c r="K48">
-        <v>0.28199999999999997</v>
+        <v>0.282</v>
       </c>
       <c r="L48">
-        <v>0.34499999999999997</v>
+        <v>0.345</v>
       </c>
       <c r="M48">
-        <v>1.2529999999999999</v>
+        <v>1.253</v>
       </c>
       <c r="N48">
         <v>96</v>
@@ -2195,7 +2173,7 @@
         <v>16943.52</v>
       </c>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="49">
       <c r="A49">
         <v>1997</v>
       </c>
@@ -2203,31 +2181,31 @@
         <v>24455.99</v>
       </c>
       <c r="C49">
-        <v>130.96299999999999</v>
+        <v>130.963</v>
       </c>
       <c r="E49">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="F49">
-        <v>0.33100000000000002</v>
+        <v>0.331</v>
       </c>
       <c r="G49">
-        <v>0.94199999999999995</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="H49">
         <v>1935</v>
       </c>
       <c r="I49">
-        <v>130.96299999999999</v>
+        <v>130.963</v>
       </c>
       <c r="K49">
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="L49">
-        <v>0.33100000000000002</v>
+        <v>0.331</v>
       </c>
       <c r="M49">
-        <v>0.58499999999999996</v>
+        <v>0.585</v>
       </c>
       <c r="N49">
         <v>468</v>
@@ -2236,7 +2214,7 @@
         <v>22052.99</v>
       </c>
     </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="50">
       <c r="A50">
         <v>1998</v>
       </c>
@@ -2244,25 +2222,25 @@
         <v>16861.5</v>
       </c>
       <c r="C50">
-        <v>130.42400000000001</v>
+        <v>130.424</v>
       </c>
       <c r="E50">
-        <v>0.22500000000000001</v>
+        <v>0.225</v>
       </c>
       <c r="F50">
         <v>0.3</v>
       </c>
       <c r="G50">
-        <v>0.92400000000000004</v>
+        <v>0.924</v>
       </c>
       <c r="H50">
         <v>1237</v>
       </c>
       <c r="I50">
-        <v>130.42400000000001</v>
+        <v>130.424</v>
       </c>
       <c r="K50">
-        <v>0.22500000000000001</v>
+        <v>0.225</v>
       </c>
       <c r="L50">
         <v>0.3</v>
@@ -2277,7 +2255,7 @@
         <v>14529.5</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="51">
       <c r="A51">
         <v>1999</v>
       </c>
@@ -2285,7 +2263,7 @@
         <v>22340.51</v>
       </c>
       <c r="C51">
-        <v>121.89700000000001</v>
+        <v>121.897</v>
       </c>
       <c r="E51">
         <v>0.251</v>
@@ -2294,13 +2272,13 @@
         <v>0.2</v>
       </c>
       <c r="G51">
-        <v>0.92300000000000004</v>
+        <v>0.923</v>
       </c>
       <c r="H51">
         <v>1085</v>
       </c>
       <c r="I51">
-        <v>121.89700000000001</v>
+        <v>121.897</v>
       </c>
       <c r="K51">
         <v>0.251</v>
@@ -2309,33 +2287,33 @@
         <v>0.2</v>
       </c>
       <c r="M51">
-        <v>2.1030000000000002</v>
+        <v>2.103</v>
       </c>
       <c r="N51">
         <v>3333</v>
       </c>
       <c r="T51">
-        <v>17922.509999999998</v>
-      </c>
-    </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.35">
+        <v>17922.51</v>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52">
         <v>2000</v>
       </c>
       <c r="B52">
-        <v>28945.602999999999</v>
+        <v>28945.603</v>
       </c>
       <c r="C52">
         <v>117.292</v>
       </c>
       <c r="E52">
-        <v>0.29799999999999999</v>
+        <v>0.298</v>
       </c>
       <c r="F52">
         <v>0.187</v>
       </c>
       <c r="G52">
-        <v>0.92700000000000005</v>
+        <v>0.927</v>
       </c>
       <c r="H52">
         <v>1423</v>
@@ -2344,7 +2322,7 @@
         <v>117.292</v>
       </c>
       <c r="K52">
-        <v>0.29799999999999999</v>
+        <v>0.298</v>
       </c>
       <c r="L52">
         <v>0.187</v>
@@ -2356,18 +2334,18 @@
         <v>3369</v>
       </c>
       <c r="T52">
-        <v>24153.602999999999</v>
+        <v>24153.603</v>
       </c>
       <c r="Y52">
         <v>1.075</v>
       </c>
     </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="53">
       <c r="A53">
         <v>2001</v>
       </c>
       <c r="B53">
-        <v>21181.764999999999</v>
+        <v>21181.765</v>
       </c>
       <c r="C53">
         <v>129.786</v>
@@ -2376,10 +2354,10 @@
         <v>0.246</v>
       </c>
       <c r="F53">
-        <v>0.26800000000000002</v>
+        <v>0.268</v>
       </c>
       <c r="G53">
-        <v>0.86199999999999999</v>
+        <v>0.862</v>
       </c>
       <c r="H53">
         <v>1058</v>
@@ -2391,10 +2369,10 @@
         <v>0.246</v>
       </c>
       <c r="L53">
-        <v>0.26800000000000002</v>
+        <v>0.268</v>
       </c>
       <c r="M53">
-        <v>1.1910000000000001</v>
+        <v>1.191</v>
       </c>
       <c r="N53">
         <v>1701</v>
@@ -2403,27 +2381,27 @@
         <v>1.157</v>
       </c>
       <c r="T53">
-        <v>18422.764999999999</v>
+        <v>18422.765</v>
       </c>
       <c r="Y53">
-        <v>1.1870000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.187</v>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54">
         <v>2002</v>
       </c>
       <c r="B54">
-        <v>26016.432000000001</v>
+        <v>26016.432</v>
       </c>
       <c r="C54">
         <v>165.142</v>
       </c>
       <c r="E54">
-        <v>0.22600000000000001</v>
+        <v>0.226</v>
       </c>
       <c r="F54">
-        <v>0.59299999999999997</v>
+        <v>0.593</v>
       </c>
       <c r="G54">
         <v>0.87</v>
@@ -2435,45 +2413,45 @@
         <v>120.429</v>
       </c>
       <c r="K54">
-        <v>0.26500000000000001</v>
+        <v>0.265</v>
       </c>
       <c r="L54">
         <v>0.215</v>
       </c>
       <c r="M54">
-        <v>1.3220000000000001</v>
+        <v>1.322</v>
       </c>
       <c r="N54">
         <v>4520</v>
       </c>
       <c r="S54">
-        <v>1.0549999999999999</v>
+        <v>1.055</v>
       </c>
       <c r="T54">
-        <v>20450.432000000001</v>
+        <v>20450.432</v>
       </c>
       <c r="U54">
-        <v>209.85599999999999</v>
+        <v>209.856</v>
       </c>
       <c r="W54">
         <v>0.186</v>
       </c>
       <c r="X54">
-        <v>0.97099999999999997</v>
+        <v>0.971</v>
       </c>
       <c r="Y54">
         <v>1.117</v>
       </c>
     </row>
-    <row r="55" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="55">
       <c r="A55">
         <v>2003</v>
       </c>
       <c r="B55">
-        <v>33361.798000000003</v>
+        <v>33361.798</v>
       </c>
       <c r="C55">
-        <v>160.28800000000001</v>
+        <v>160.288</v>
       </c>
       <c r="E55">
         <v>0.122</v>
@@ -2482,16 +2460,16 @@
         <v>0.65</v>
       </c>
       <c r="G55">
-        <v>0.86599999999999999</v>
+        <v>0.866</v>
       </c>
       <c r="H55">
         <v>1157</v>
       </c>
       <c r="I55">
-        <v>130.57599999999999</v>
+        <v>130.576</v>
       </c>
       <c r="K55">
-        <v>0.24299999999999999</v>
+        <v>0.243</v>
       </c>
       <c r="L55">
         <v>0.3</v>
@@ -2506,7 +2484,7 @@
         <v>1.139</v>
       </c>
       <c r="T55">
-        <v>24936.797999999999</v>
+        <v>24936.798</v>
       </c>
       <c r="U55">
         <v>190</v>
@@ -2518,39 +2496,39 @@
         <v>1</v>
       </c>
       <c r="Y55">
-        <v>1.1120000000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.35">
+        <v>1.112</v>
+      </c>
+    </row>
+    <row r="56">
       <c r="A56">
         <v>2004</v>
       </c>
       <c r="B56">
-        <v>40935.357000000004</v>
+        <v>40935.357</v>
       </c>
       <c r="C56">
         <v>161.298</v>
       </c>
       <c r="E56">
-        <v>0.26600000000000001</v>
+        <v>0.266</v>
       </c>
       <c r="F56">
-        <v>0.60899999999999999</v>
+        <v>0.609</v>
       </c>
       <c r="G56">
-        <v>0.88600000000000001</v>
+        <v>0.886</v>
       </c>
       <c r="H56">
         <v>1132</v>
       </c>
       <c r="I56">
-        <v>137.86000000000001</v>
+        <v>137.86</v>
       </c>
       <c r="K56">
-        <v>0.27900000000000003</v>
+        <v>0.279</v>
       </c>
       <c r="L56">
-        <v>0.38300000000000001</v>
+        <v>0.383</v>
       </c>
       <c r="M56">
         <v>0.747</v>
@@ -2559,42 +2537,42 @@
         <v>7298</v>
       </c>
       <c r="S56">
-        <v>1.0049999999999999</v>
+        <v>1.005</v>
       </c>
       <c r="T56">
         <v>32505.357</v>
       </c>
       <c r="U56">
-        <v>184.73500000000001</v>
+        <v>184.735</v>
       </c>
       <c r="W56">
         <v>0.253</v>
       </c>
       <c r="X56">
-        <v>0.83499999999999996</v>
+        <v>0.835</v>
       </c>
       <c r="Y56">
-        <v>0.84199999999999997</v>
-      </c>
-    </row>
-    <row r="57" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.842</v>
+      </c>
+    </row>
+    <row r="57">
       <c r="A57">
         <v>2005</v>
       </c>
       <c r="B57">
-        <v>43858.196000000004</v>
+        <v>43858.196</v>
       </c>
       <c r="C57">
-        <v>182.59299999999999</v>
+        <v>182.593</v>
       </c>
       <c r="E57">
-        <v>0.23899999999999999</v>
+        <v>0.239</v>
       </c>
       <c r="F57">
-        <v>0.73199999999999998</v>
+        <v>0.732</v>
       </c>
       <c r="G57">
-        <v>0.91800000000000004</v>
+        <v>0.918</v>
       </c>
       <c r="H57">
         <v>1019</v>
@@ -2603,13 +2581,13 @@
         <v>138.184</v>
       </c>
       <c r="K57">
-        <v>0.27800000000000002</v>
+        <v>0.278</v>
       </c>
       <c r="L57">
-        <v>0.40300000000000002</v>
+        <v>0.403</v>
       </c>
       <c r="M57">
-        <v>0.93200000000000005</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="N57">
         <v>6599</v>
@@ -2618,7 +2596,7 @@
         <v>0.89</v>
       </c>
       <c r="T57">
-        <v>36240.196000000004</v>
+        <v>36240.196</v>
       </c>
       <c r="U57">
         <v>204.798</v>
@@ -2627,13 +2605,13 @@
         <v>0.219</v>
       </c>
       <c r="X57">
-        <v>0.89600000000000002</v>
+        <v>0.896</v>
       </c>
       <c r="Y57">
-        <v>0.79200000000000004</v>
-      </c>
-    </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.792</v>
+      </c>
+    </row>
+    <row r="58">
       <c r="A58">
         <v>2006</v>
       </c>
@@ -2644,13 +2622,13 @@
         <v>185.51</v>
       </c>
       <c r="E58">
-        <v>0.19600000000000001</v>
+        <v>0.196</v>
       </c>
       <c r="F58">
-        <v>0.74199999999999999</v>
+        <v>0.742</v>
       </c>
       <c r="G58">
-        <v>0.93799999999999994</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="H58">
         <v>1081</v>
@@ -2659,54 +2637,54 @@
         <v>144.917</v>
       </c>
       <c r="K58">
-        <v>0.24199999999999999</v>
+        <v>0.242</v>
       </c>
       <c r="L58">
-        <v>0.55100000000000005</v>
+        <v>0.551</v>
       </c>
       <c r="M58">
-        <v>0.65500000000000003</v>
+        <v>0.655</v>
       </c>
       <c r="N58">
         <v>6797</v>
       </c>
       <c r="S58">
-        <v>0.82199999999999995</v>
+        <v>0.822</v>
       </c>
       <c r="T58">
         <v>32712.555</v>
       </c>
       <c r="U58">
-        <v>205.80600000000001</v>
+        <v>205.806</v>
       </c>
       <c r="W58">
-        <v>0.17299999999999999</v>
+        <v>0.173</v>
       </c>
       <c r="X58">
-        <v>0.83799999999999997</v>
+        <v>0.838</v>
       </c>
       <c r="Y58">
-        <v>0.89200000000000002</v>
-      </c>
-    </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.892</v>
+      </c>
+    </row>
+    <row r="59">
       <c r="A59">
         <v>2007</v>
       </c>
       <c r="B59">
-        <v>38639.050999999999</v>
+        <v>38639.051</v>
       </c>
       <c r="C59">
-        <v>167.86099999999999</v>
+        <v>167.861</v>
       </c>
       <c r="E59">
-        <v>0.25600000000000001</v>
+        <v>0.256</v>
       </c>
       <c r="F59">
-        <v>0.61399999999999999</v>
+        <v>0.614</v>
       </c>
       <c r="G59">
-        <v>0.93300000000000005</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="H59">
         <v>1333</v>
@@ -2718,34 +2696,34 @@
         <v>0.31</v>
       </c>
       <c r="L59">
-        <v>0.29799999999999999</v>
+        <v>0.298</v>
       </c>
       <c r="M59">
-        <v>0.91700000000000004</v>
+        <v>0.917</v>
       </c>
       <c r="N59">
         <v>5758</v>
       </c>
       <c r="S59">
-        <v>0.86099999999999999</v>
+        <v>0.861</v>
       </c>
       <c r="T59">
-        <v>31548.050999999999</v>
+        <v>31548.051</v>
       </c>
       <c r="U59">
-        <v>182.32599999999999</v>
+        <v>182.326</v>
       </c>
       <c r="W59">
-        <v>0.23799999999999999</v>
+        <v>0.238</v>
       </c>
       <c r="X59">
-        <v>0.71899999999999997</v>
+        <v>0.719</v>
       </c>
       <c r="Y59">
-        <v>0.98299999999999998</v>
-      </c>
-    </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.983</v>
+      </c>
+    </row>
+    <row r="60">
       <c r="A60">
         <v>2008</v>
       </c>
@@ -2759,66 +2737,66 @@
         <v>0.19</v>
       </c>
       <c r="F60">
-        <v>0.70099999999999996</v>
+        <v>0.701</v>
       </c>
       <c r="G60">
-        <v>0.91500000000000004</v>
+        <v>0.915</v>
       </c>
       <c r="H60">
         <v>2829</v>
       </c>
       <c r="I60">
-        <v>142.08000000000001</v>
+        <v>142.08</v>
       </c>
       <c r="K60">
-        <v>0.16600000000000001</v>
+        <v>0.166</v>
       </c>
       <c r="L60">
-        <v>0.38600000000000001</v>
+        <v>0.386</v>
       </c>
       <c r="M60">
-        <v>0.84899999999999998</v>
+        <v>0.849</v>
       </c>
       <c r="N60">
         <v>6139</v>
       </c>
       <c r="S60">
-        <v>0.94699999999999995</v>
+        <v>0.947</v>
       </c>
       <c r="T60">
         <v>33555.642</v>
       </c>
       <c r="U60">
-        <v>194.78899999999999</v>
+        <v>194.789</v>
       </c>
       <c r="W60">
-        <v>0.20300000000000001</v>
+        <v>0.203</v>
       </c>
       <c r="X60">
-        <v>0.85899999999999999</v>
+        <v>0.859</v>
       </c>
       <c r="Y60">
-        <v>0.82199999999999995</v>
-      </c>
-    </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.822</v>
+      </c>
+    </row>
+    <row r="61">
       <c r="A61">
         <v>2009</v>
       </c>
       <c r="B61">
-        <v>48428.983999999997</v>
+        <v>48428.984</v>
       </c>
       <c r="C61">
-        <v>181.24700000000001</v>
+        <v>181.247</v>
       </c>
       <c r="E61">
-        <v>0.20399999999999999</v>
+        <v>0.204</v>
       </c>
       <c r="F61">
         <v>0.79</v>
       </c>
       <c r="G61">
-        <v>0.88600000000000001</v>
+        <v>0.886</v>
       </c>
       <c r="H61">
         <v>3215</v>
@@ -2830,7 +2808,7 @@
         <v>0.249</v>
       </c>
       <c r="L61">
-        <v>0.40400000000000003</v>
+        <v>0.404</v>
       </c>
       <c r="M61">
         <v>1.518</v>
@@ -2839,39 +2817,39 @@
         <v>5263</v>
       </c>
       <c r="O61">
-        <v>194.13300000000001</v>
+        <v>194.133</v>
       </c>
       <c r="Q61">
         <v>0.153</v>
       </c>
       <c r="R61">
-        <v>0.95499999999999996</v>
+        <v>0.955</v>
       </c>
       <c r="S61">
-        <v>1.0409999999999999</v>
+        <v>1.041</v>
       </c>
       <c r="T61">
-        <v>39950.983999999997</v>
+        <v>39950.984</v>
       </c>
       <c r="U61">
         <v>196.738</v>
       </c>
       <c r="W61">
-        <v>0.20599999999999999</v>
+        <v>0.206</v>
       </c>
       <c r="X61">
         <v>0.9</v>
       </c>
       <c r="Y61">
-        <v>0.67200000000000004</v>
-      </c>
-    </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.672</v>
+      </c>
+    </row>
+    <row r="62">
       <c r="A62">
         <v>2010</v>
       </c>
       <c r="B62">
-        <v>46505.906000000003</v>
+        <v>46505.906</v>
       </c>
       <c r="C62">
         <v>171.405</v>
@@ -2880,34 +2858,34 @@
         <v>0.218</v>
       </c>
       <c r="F62">
-        <v>0.71599999999999997</v>
+        <v>0.716</v>
       </c>
       <c r="G62">
-        <v>0.85099999999999998</v>
+        <v>0.851</v>
       </c>
       <c r="H62">
         <v>2071</v>
       </c>
       <c r="I62">
-        <v>156.21600000000001</v>
+        <v>156.216</v>
       </c>
       <c r="K62">
         <v>0.26</v>
       </c>
       <c r="L62">
-        <v>0.57499999999999996</v>
+        <v>0.575</v>
       </c>
       <c r="M62">
-        <v>0.54100000000000004</v>
+        <v>0.541</v>
       </c>
       <c r="N62">
         <v>4065</v>
       </c>
       <c r="O62">
-        <v>200.52799999999999</v>
+        <v>200.528</v>
       </c>
       <c r="Q62">
-        <v>0.13200000000000001</v>
+        <v>0.132</v>
       </c>
       <c r="R62">
         <v>0.98</v>
@@ -2916,39 +2894,39 @@
         <v>1.155</v>
       </c>
       <c r="T62">
-        <v>40369.906000000003</v>
+        <v>40369.906</v>
       </c>
       <c r="U62">
         <v>166.76</v>
       </c>
       <c r="W62">
-        <v>0.23300000000000001</v>
+        <v>0.233</v>
       </c>
       <c r="X62">
-        <v>0.67600000000000005</v>
+        <v>0.676</v>
       </c>
       <c r="Y62">
-        <v>0.77900000000000003</v>
-      </c>
-    </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.779</v>
+      </c>
+    </row>
+    <row r="63">
       <c r="A63">
         <v>2011</v>
       </c>
       <c r="B63">
-        <v>48861.785000000003</v>
+        <v>48861.785</v>
       </c>
       <c r="C63">
-        <v>189.49100000000001</v>
+        <v>189.491</v>
       </c>
       <c r="E63">
         <v>0.155</v>
       </c>
       <c r="F63">
-        <v>0.83799999999999997</v>
+        <v>0.838</v>
       </c>
       <c r="G63">
-        <v>0.81599999999999995</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="H63">
         <v>1963</v>
@@ -2960,16 +2938,16 @@
         <v>0.219</v>
       </c>
       <c r="L63">
-        <v>0.35699999999999998</v>
+        <v>0.357</v>
       </c>
       <c r="M63">
-        <v>0.67700000000000005</v>
+        <v>0.677</v>
       </c>
       <c r="N63">
         <v>5022</v>
       </c>
       <c r="O63">
-        <v>203.33600000000001</v>
+        <v>203.336</v>
       </c>
       <c r="Q63">
         <v>0.129</v>
@@ -2978,42 +2956,42 @@
         <v>0.99</v>
       </c>
       <c r="S63">
-        <v>1.0740000000000001</v>
+        <v>1.074</v>
       </c>
       <c r="T63">
-        <v>41876.785000000003</v>
+        <v>41876.785</v>
       </c>
       <c r="U63">
-        <v>201.98099999999999</v>
+        <v>201.981</v>
       </c>
       <c r="W63">
-        <v>0.14299999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="X63">
-        <v>0.94699999999999995</v>
+        <v>0.947</v>
       </c>
       <c r="Y63">
-        <v>0.65600000000000003</v>
-      </c>
-    </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.656</v>
+      </c>
+    </row>
+    <row r="64">
       <c r="A64">
         <v>2012</v>
       </c>
       <c r="B64">
-        <v>52250.358999999997</v>
+        <v>52250.359</v>
       </c>
       <c r="C64">
-        <v>184.49600000000001</v>
+        <v>184.496</v>
       </c>
       <c r="E64">
         <v>0.2</v>
       </c>
       <c r="F64">
-        <v>0.84499999999999997</v>
+        <v>0.845</v>
       </c>
       <c r="G64">
-        <v>0.77800000000000002</v>
+        <v>0.778</v>
       </c>
       <c r="H64">
         <v>2267</v>
@@ -3022,13 +3000,13 @@
         <v>178.834</v>
       </c>
       <c r="K64">
-        <v>0.20799999999999999</v>
+        <v>0.208</v>
       </c>
       <c r="L64">
-        <v>0.81799999999999995</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="M64">
-        <v>0.84199999999999997</v>
+        <v>0.842</v>
       </c>
       <c r="N64">
         <v>7098</v>
@@ -3043,75 +3021,75 @@
         <v>0.96</v>
       </c>
       <c r="S64">
-        <v>1.1140000000000001</v>
+        <v>1.114</v>
       </c>
       <c r="T64">
-        <v>42885.358999999997</v>
+        <v>42885.359</v>
       </c>
       <c r="U64">
-        <v>179.09100000000001</v>
+        <v>179.091</v>
       </c>
       <c r="W64">
-        <v>0.20200000000000001</v>
+        <v>0.202</v>
       </c>
       <c r="X64">
-        <v>0.82299999999999995</v>
+        <v>0.823</v>
       </c>
       <c r="Y64">
-        <v>0.78600000000000003</v>
-      </c>
-    </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.786</v>
+      </c>
+    </row>
+    <row r="65">
       <c r="A65">
         <v>2013</v>
       </c>
       <c r="B65">
-        <v>56494.726999999999</v>
+        <v>56494.727</v>
       </c>
       <c r="C65">
-        <v>173.03700000000001</v>
+        <v>173.037</v>
       </c>
       <c r="E65">
-        <v>0.22800000000000001</v>
+        <v>0.228</v>
       </c>
       <c r="F65">
-        <v>0.71299999999999997</v>
+        <v>0.713</v>
       </c>
       <c r="G65">
-        <v>0.75800000000000001</v>
+        <v>0.758</v>
       </c>
       <c r="H65">
         <v>1840</v>
       </c>
       <c r="I65">
-        <v>146.24799999999999</v>
+        <v>146.248</v>
       </c>
       <c r="K65">
-        <v>0.28399999999999997</v>
+        <v>0.284</v>
       </c>
       <c r="L65">
         <v>0.432</v>
       </c>
       <c r="M65">
-        <v>0.46899999999999997</v>
+        <v>0.469</v>
       </c>
       <c r="N65">
         <v>8116</v>
       </c>
       <c r="O65">
-        <v>197.13399999999999</v>
+        <v>197.134</v>
       </c>
       <c r="Q65">
-        <v>0.19900000000000001</v>
+        <v>0.199</v>
       </c>
       <c r="R65">
         <v>0.86</v>
       </c>
       <c r="S65">
-        <v>0.91700000000000004</v>
+        <v>0.917</v>
       </c>
       <c r="T65">
-        <v>46538.726999999999</v>
+        <v>46538.727</v>
       </c>
       <c r="U65">
         <v>173.71</v>
@@ -3123,10 +3101,10 @@
         <v>0.746</v>
       </c>
       <c r="Y65">
-        <v>0.79200000000000004</v>
-      </c>
-    </row>
-    <row r="66" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.792</v>
+      </c>
+    </row>
+    <row r="66">
       <c r="A66">
         <v>2014</v>
       </c>
@@ -3134,55 +3112,55 @@
         <v>54756.72</v>
       </c>
       <c r="C66">
-        <v>172.56299999999999</v>
+        <v>172.563</v>
       </c>
       <c r="E66">
-        <v>0.19600000000000001</v>
+        <v>0.196</v>
       </c>
       <c r="F66">
-        <v>0.77700000000000002</v>
+        <v>0.777</v>
       </c>
       <c r="G66">
-        <v>0.70799999999999996</v>
+        <v>0.708</v>
       </c>
       <c r="H66">
         <v>1491</v>
       </c>
       <c r="M66">
-        <v>0.66400000000000003</v>
+        <v>0.664</v>
       </c>
       <c r="N66">
         <v>8371</v>
       </c>
       <c r="O66">
-        <v>183.93299999999999</v>
+        <v>183.933</v>
       </c>
       <c r="Q66">
-        <v>0.16700000000000001</v>
+        <v>0.167</v>
       </c>
       <c r="R66">
         <v>0.876</v>
       </c>
       <c r="S66">
-        <v>0.80800000000000005</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="T66">
-        <v>44894.720000000001</v>
+        <v>44894.72</v>
       </c>
       <c r="U66">
         <v>169.72</v>
       </c>
       <c r="W66">
-        <v>0.20300000000000001</v>
+        <v>0.203</v>
       </c>
       <c r="X66">
         <v>0.753</v>
       </c>
       <c r="Y66">
-        <v>0.74199999999999999</v>
-      </c>
-    </row>
-    <row r="67" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.742</v>
+      </c>
+    </row>
+    <row r="67">
       <c r="A67">
         <v>2015</v>
       </c>
@@ -3190,16 +3168,16 @@
         <v>50794.01</v>
       </c>
       <c r="C67">
-        <v>180.40600000000001</v>
+        <v>180.406</v>
       </c>
       <c r="E67">
-        <v>0.19900000000000001</v>
+        <v>0.199</v>
       </c>
       <c r="F67">
         <v>0.73</v>
       </c>
       <c r="G67">
-        <v>0.67900000000000005</v>
+        <v>0.679</v>
       </c>
       <c r="H67">
         <v>1503</v>
@@ -3208,7 +3186,7 @@
         <v>138.827</v>
       </c>
       <c r="K67">
-        <v>0.26800000000000002</v>
+        <v>0.268</v>
       </c>
       <c r="L67">
         <v>0.378</v>
@@ -3223,19 +3201,19 @@
         <v>189.238</v>
       </c>
       <c r="Q67">
-        <v>0.17599999999999999</v>
+        <v>0.176</v>
       </c>
       <c r="R67">
-        <v>0.88300000000000001</v>
+        <v>0.883</v>
       </c>
       <c r="S67">
-        <v>0.94299999999999995</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="T67">
         <v>42886.01</v>
       </c>
       <c r="U67">
-        <v>188.59299999999999</v>
+        <v>188.593</v>
       </c>
       <c r="W67">
         <v>0.187</v>
@@ -3244,10 +3222,10 @@
         <v>0.78</v>
       </c>
       <c r="Y67">
-        <v>0.95299999999999996</v>
-      </c>
-    </row>
-    <row r="68" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.953</v>
+      </c>
+    </row>
+    <row r="68">
       <c r="A68">
         <v>2016</v>
       </c>
@@ -3255,16 +3233,16 @@
         <v>55308.288</v>
       </c>
       <c r="C68">
-        <v>189.18299999999999</v>
+        <v>189.183</v>
       </c>
       <c r="E68">
-        <v>0.22500000000000001</v>
+        <v>0.225</v>
       </c>
       <c r="F68">
-        <v>0.81799999999999995</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="G68">
-        <v>0.65400000000000003</v>
+        <v>0.654</v>
       </c>
       <c r="H68">
         <v>1167</v>
@@ -3273,10 +3251,10 @@
         <v>150.084</v>
       </c>
       <c r="K68">
-        <v>0.34599999999999997</v>
+        <v>0.346</v>
       </c>
       <c r="L68">
-        <v>0.53600000000000003</v>
+        <v>0.536</v>
       </c>
       <c r="M68">
         <v>1.077</v>
@@ -3285,13 +3263,13 @@
         <v>6272</v>
       </c>
       <c r="O68">
-        <v>180.68199999999999</v>
+        <v>180.682</v>
       </c>
       <c r="Q68">
-        <v>0.19500000000000001</v>
+        <v>0.195</v>
       </c>
       <c r="R68">
-        <v>0.85199999999999998</v>
+        <v>0.852</v>
       </c>
       <c r="S68">
         <v>1.077</v>
@@ -3300,33 +3278,33 @@
         <v>47869.288</v>
       </c>
       <c r="U68">
-        <v>212.98400000000001</v>
+        <v>212.984</v>
       </c>
       <c r="W68">
-        <v>0.17899999999999999</v>
+        <v>0.179</v>
       </c>
       <c r="X68">
-        <v>0.94199999999999995</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="Y68">
-        <v>0.98399999999999999</v>
-      </c>
-    </row>
-    <row r="69" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.984</v>
+      </c>
+    </row>
+    <row r="69">
       <c r="A69">
         <v>2017</v>
       </c>
       <c r="B69">
-        <v>57529.906999999999</v>
+        <v>57529.907</v>
       </c>
       <c r="C69">
-        <v>181.44900000000001</v>
+        <v>181.449</v>
       </c>
       <c r="E69">
         <v>0.222</v>
       </c>
       <c r="F69">
-        <v>0.70899999999999996</v>
+        <v>0.709</v>
       </c>
       <c r="G69">
         <v>0.61</v>
@@ -3335,13 +3313,13 @@
         <v>1374</v>
       </c>
       <c r="I69">
-        <v>153.08500000000001</v>
+        <v>153.085</v>
       </c>
       <c r="K69">
-        <v>0.28599999999999998</v>
+        <v>0.286</v>
       </c>
       <c r="L69">
-        <v>0.52700000000000002</v>
+        <v>0.527</v>
       </c>
       <c r="M69">
         <v>1.282</v>
@@ -3356,45 +3334,45 @@
         <v>0.223</v>
       </c>
       <c r="R69">
-        <v>0.66900000000000004</v>
+        <v>0.669</v>
       </c>
       <c r="S69">
-        <v>1.0349999999999999</v>
+        <v>1.035</v>
       </c>
       <c r="T69">
-        <v>50965.906999999999</v>
+        <v>50965.907</v>
       </c>
       <c r="U69">
         <v>189.012</v>
       </c>
       <c r="W69">
-        <v>0.20899999999999999</v>
+        <v>0.209</v>
       </c>
       <c r="X69">
         <v>0.753</v>
       </c>
       <c r="Y69">
-        <v>0.82599999999999996</v>
-      </c>
-    </row>
-    <row r="70" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.826</v>
+      </c>
+    </row>
+    <row r="70">
       <c r="A70">
         <v>2018</v>
       </c>
       <c r="B70">
-        <v>37030.906000000003</v>
+        <v>37030.906</v>
       </c>
       <c r="C70">
-        <v>170.81100000000001</v>
+        <v>170.811</v>
       </c>
       <c r="E70">
-        <v>0.23300000000000001</v>
+        <v>0.233</v>
       </c>
       <c r="F70">
-        <v>0.69599999999999995</v>
+        <v>0.696</v>
       </c>
       <c r="G70">
-        <v>0.58299999999999996</v>
+        <v>0.583</v>
       </c>
       <c r="H70">
         <v>861</v>
@@ -3415,63 +3393,63 @@
         <v>2697</v>
       </c>
       <c r="O70">
-        <v>195.59899999999999</v>
+        <v>195.599</v>
       </c>
       <c r="Q70">
-        <v>0.19500000000000001</v>
+        <v>0.195</v>
       </c>
       <c r="R70">
         <v>0.93</v>
       </c>
       <c r="S70">
-        <v>0.99299999999999999</v>
+        <v>0.993</v>
       </c>
       <c r="T70">
-        <v>33472.906000000003</v>
+        <v>33472.906</v>
       </c>
       <c r="U70">
-        <v>169.94800000000001</v>
+        <v>169.948</v>
       </c>
       <c r="W70">
-        <v>0.23799999999999999</v>
+        <v>0.238</v>
       </c>
       <c r="X70">
-        <v>0.69199999999999995</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="Y70">
-        <v>0.93400000000000005</v>
-      </c>
-    </row>
-    <row r="71" spans="1:25" x14ac:dyDescent="0.35">
+        <v>0.9340000000000001</v>
+      </c>
+    </row>
+    <row r="71">
       <c r="A71">
         <v>2019</v>
       </c>
       <c r="B71">
-        <v>43240.186999999998</v>
+        <v>43240.187</v>
       </c>
       <c r="C71">
-        <v>177.78800000000001</v>
+        <v>177.788</v>
       </c>
       <c r="E71">
-        <v>0.20399999999999999</v>
+        <v>0.204</v>
       </c>
       <c r="F71">
-        <v>0.77700000000000002</v>
+        <v>0.777</v>
       </c>
       <c r="G71">
-        <v>0.57599999999999996</v>
+        <v>0.576</v>
       </c>
       <c r="H71">
         <v>915</v>
       </c>
       <c r="I71">
-        <v>138.29900000000001</v>
+        <v>138.299</v>
       </c>
       <c r="K71">
-        <v>0.26600000000000001</v>
+        <v>0.266</v>
       </c>
       <c r="L71">
-        <v>0.41099999999999998</v>
+        <v>0.411</v>
       </c>
       <c r="M71">
         <v>1.153</v>
@@ -3483,28 +3461,28 @@
         <v>199.078</v>
       </c>
       <c r="Q71">
-        <v>0.21299999999999999</v>
+        <v>0.213</v>
       </c>
       <c r="R71">
-        <v>0.85799999999999998</v>
+        <v>0.858</v>
       </c>
       <c r="S71">
-        <v>0.96899999999999997</v>
+        <v>0.969</v>
       </c>
       <c r="T71">
-        <v>38981.186999999998</v>
+        <v>38981.187</v>
       </c>
       <c r="U71">
-        <v>182.33699999999999</v>
+        <v>182.337</v>
       </c>
       <c r="W71">
         <v>0.186</v>
       </c>
       <c r="X71">
-        <v>0.84799999999999998</v>
+        <v>0.848</v>
       </c>
       <c r="Y71">
-        <v>0.84399999999999997</v>
+        <v>0.844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>